<commit_message>
Support SWay layout and wrap selected FPT pairs
</commit_message>
<xml_diff>
--- a/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
+++ b/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
@@ -413,647 +413,777 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Pair_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Pair_Label</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>RPM</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Diesel_Speed_RPM</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Diesel_Power_kW</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Diesel_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Diesel_Consumo_L_h</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Diesel_Custo_R_h</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1100</v>
       </c>
-      <c r="B2" t="n">
+      <c r="D2" t="n">
         <v>1100.019</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>101.5714</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>21.938</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>25.71864009378664</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>138.8806565064478</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="H2" t="n">
+      <c r="J2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>100.54</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>40.794</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>-23.75255350293668</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>1200</v>
       </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
         <v>1199.906</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>112.8476</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>24.062</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>28.20867526377491</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>152.3268464243845</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>43.955</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>-25.09641461978385</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>1300</v>
       </c>
-      <c r="B4" t="n">
+      <c r="D4" t="n">
         <v>1300</v>
       </c>
-      <c r="C4" t="n">
+      <c r="E4" t="n">
         <v>126.6131</v>
       </c>
-      <c r="D4" t="n">
+      <c r="F4" t="n">
         <v>26.415</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>30.96717467760844</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>167.2227432590856</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>47.414</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="M4" t="n">
+      <c r="O4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>-26.39928644672269</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>1400</v>
       </c>
-      <c r="B5" t="n">
+      <c r="D5" t="n">
         <v>1400.01</v>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>142.0559</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>29.065</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>34.07385697538101</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>183.9988276670574</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="H5" t="n">
+      <c r="J5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>135.548</v>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>51.639</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="M5" t="n">
+      <c r="O5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>-27.14933161687878</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>1500</v>
       </c>
-      <c r="B6" t="n">
+      <c r="D6" t="n">
         <v>1500.01</v>
       </c>
-      <c r="C6" t="n">
+      <c r="E6" t="n">
         <v>158.5028</v>
       </c>
-      <c r="D6" t="n">
+      <c r="F6" t="n">
         <v>32.921</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>38.59437280187574</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>208.409613130129</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="H6" t="n">
+      <c r="J6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="J6" t="n">
+      <c r="L6" t="n">
         <v>58.213</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>-27.49415690300805</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>1600</v>
       </c>
-      <c r="B7" t="n">
+      <c r="D7" t="n">
         <v>1600.044</v>
       </c>
-      <c r="C7" t="n">
+      <c r="E7" t="n">
         <v>168.0404</v>
       </c>
-      <c r="D7" t="n">
+      <c r="F7" t="n">
         <v>34.72</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>40.70339976553341</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>219.7983587338804</v>
       </c>
-      <c r="G7" t="n">
+      <c r="I7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="H7" t="n">
+      <c r="J7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="J7" t="n">
+      <c r="L7" t="n">
         <v>62.66</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>-25.99914824709473</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>1700</v>
       </c>
-      <c r="B8" t="n">
+      <c r="D8" t="n">
         <v>1699.996</v>
       </c>
-      <c r="C8" t="n">
+      <c r="E8" t="n">
         <v>178.8622</v>
       </c>
-      <c r="D8" t="n">
+      <c r="F8" t="n">
         <v>36.915</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>43.27667057444314</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>233.694021101993</v>
       </c>
-      <c r="G8" t="n">
+      <c r="I8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="H8" t="n">
+      <c r="J8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="J8" t="n">
+      <c r="L8" t="n">
         <v>65.848</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>-26.85818039909983</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>1800</v>
       </c>
-      <c r="B9" t="n">
+      <c r="D9" t="n">
         <v>1799.969</v>
       </c>
-      <c r="C9" t="n">
+      <c r="E9" t="n">
         <v>189.4811</v>
       </c>
-      <c r="D9" t="n">
+      <c r="F9" t="n">
         <v>39.393</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>46.18171160609613</v>
       </c>
-      <c r="F9" t="n">
+      <c r="H9" t="n">
         <v>249.3812426729191</v>
       </c>
-      <c r="G9" t="n">
+      <c r="I9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="H9" t="n">
+      <c r="J9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="J9" t="n">
+      <c r="L9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>-30.32976437212198</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>1900</v>
       </c>
-      <c r="B10" t="n">
+      <c r="D10" t="n">
         <v>1899.985</v>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>199.5484</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
         <v>41.813</v>
       </c>
-      <c r="E10" t="n">
+      <c r="G10" t="n">
         <v>49.01875732708089</v>
       </c>
-      <c r="F10" t="n">
+      <c r="H10" t="n">
         <v>264.7012895662368</v>
       </c>
-      <c r="G10" t="n">
+      <c r="I10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="H10" t="n">
+      <c r="J10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>180.749</v>
       </c>
-      <c r="J10" t="n">
+      <c r="L10" t="n">
         <v>68.246</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>-33.07445479329911</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>2000</v>
       </c>
-      <c r="B11" t="n">
+      <c r="D11" t="n">
         <v>1999.993</v>
       </c>
-      <c r="C11" t="n">
+      <c r="E11" t="n">
         <v>205.9202</v>
       </c>
-      <c r="D11" t="n">
+      <c r="F11" t="n">
         <v>43.791</v>
       </c>
-      <c r="E11" t="n">
+      <c r="G11" t="n">
         <v>51.33763188745603</v>
       </c>
-      <c r="F11" t="n">
+      <c r="H11" t="n">
         <v>277.2232121922626</v>
       </c>
-      <c r="G11" t="n">
+      <c r="I11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="H11" t="n">
+      <c r="J11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="J11" t="n">
+      <c r="L11" t="n">
         <v>67.595</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>-36.70698936277493</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
         <v>2100</v>
       </c>
-      <c r="B12" t="n">
+      <c r="D12" t="n">
         <v>2100.011</v>
       </c>
-      <c r="C12" t="n">
+      <c r="E12" t="n">
         <v>190.74</v>
       </c>
-      <c r="D12" t="n">
+      <c r="F12" t="n">
         <v>40.444</v>
       </c>
-      <c r="E12" t="n">
+      <c r="G12" t="n">
         <v>47.41383352872216</v>
       </c>
-      <c r="F12" t="n">
+      <c r="H12" t="n">
         <v>256.0347010550997</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="H12" t="n">
+      <c r="J12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="I12" t="n">
+      <c r="K12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="J12" t="n">
+      <c r="L12" t="n">
         <v>67.64</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>-31.42346434456669</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>P241075_NEF6_HORSCH_FULL_LOAD_CURVE_SALA01_PUC MINAS_D85B15 vs P251122_NEF67_175KW_MAR_l_SN2040912_Full_Load_Curve_rev24_E94H6</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
         <v>2200</v>
       </c>
-      <c r="B13" t="n">
+      <c r="D13" t="n">
         <v>2199.961</v>
       </c>
-      <c r="C13" t="n">
+      <c r="E13" t="n">
         <v>180.1196</v>
       </c>
-      <c r="D13" t="n">
+      <c r="F13" t="n">
         <v>39.015</v>
       </c>
-      <c r="E13" t="n">
+      <c r="G13" t="n">
         <v>45.73856975381008</v>
       </c>
-      <c r="F13" t="n">
+      <c r="H13" t="n">
         <v>246.9882766705745</v>
       </c>
-      <c r="G13" t="n">
+      <c r="I13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="H13" t="n">
+      <c r="J13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="J13" t="n">
+      <c r="L13" t="n">
         <v>68.863</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>-27.62636731462547</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust FPT engine displacement by file name
</commit_message>
<xml_diff>
--- a/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
+++ b/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE23"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,7 +615,7 @@
         <v>855.284</v>
       </c>
       <c r="M2" t="n">
-        <v>85.76093459672069</v>
+        <v>165.1217994474175</v>
       </c>
       <c r="N2" t="n">
         <v>7.371469710110599</v>
@@ -651,7 +651,7 @@
         <v>614.033</v>
       </c>
       <c r="Y2" t="n">
-        <v>71.93240293527499</v>
+        <v>138.4967160992609</v>
       </c>
       <c r="Z2" t="n">
         <v>5.123065851202532</v>
@@ -714,7 +714,7 @@
         <v>1001.307</v>
       </c>
       <c r="M3" t="n">
-        <v>90.16074520659268</v>
+        <v>173.5930765917979</v>
       </c>
       <c r="N3" t="n">
         <v>9.478317989122266</v>
@@ -750,7 +750,7 @@
         <v>598.8225</v>
       </c>
       <c r="Y3" t="n">
-        <v>70.63183398702874</v>
+        <v>135.9926355869658</v>
       </c>
       <c r="Z3" t="n">
         <v>5.277530107879249</v>
@@ -813,7 +813,7 @@
         <v>1151.256</v>
       </c>
       <c r="M4" t="n">
-        <v>94.87618551787044</v>
+        <v>182.672058683661</v>
       </c>
       <c r="N4" t="n">
         <v>12.20416552876442</v>
@@ -849,7 +849,7 @@
         <v>618.6754</v>
       </c>
       <c r="Y4" t="n">
-        <v>71.49738164776328</v>
+        <v>137.6591377994248</v>
       </c>
       <c r="Z4" t="n">
         <v>5.953061266356182</v>
@@ -912,7 +912,7 @@
         <v>1333.037</v>
       </c>
       <c r="M5" t="n">
-        <v>100.0868527420609</v>
+        <v>192.7045373690426</v>
       </c>
       <c r="N5" t="n">
         <v>15.7296847843975</v>
@@ -948,7 +948,7 @@
         <v>645.2624999999999</v>
       </c>
       <c r="Y5" t="n">
-        <v>72.01830624666327</v>
+        <v>138.6621120271576</v>
       </c>
       <c r="Z5" t="n">
         <v>6.691189980673633</v>
@@ -1011,7 +1011,7 @@
         <v>1638.823</v>
       </c>
       <c r="M6" t="n">
-        <v>109.7015870271678</v>
+        <v>211.2164884552933</v>
       </c>
       <c r="N6" t="n">
         <v>22.0044045378286</v>
@@ -1047,7 +1047,7 @@
         <v>706.9007</v>
       </c>
       <c r="Y6" t="n">
-        <v>75.58050048948876</v>
+        <v>145.520665121553</v>
       </c>
       <c r="Z6" t="n">
         <v>8.086896229873149</v>
@@ -1110,7 +1110,7 @@
         <v>1713.213</v>
       </c>
       <c r="M7" t="n">
-        <v>108.7813121895017</v>
+        <v>209.4446160066526</v>
       </c>
       <c r="N7" t="n">
         <v>24.09184179296887</v>
@@ -1146,7 +1146,7 @@
         <v>720.8134</v>
       </c>
       <c r="Y7" t="n">
-        <v>74.81759260933984</v>
+        <v>144.0517827851469</v>
       </c>
       <c r="Z7" t="n">
         <v>8.844545266070686</v>
@@ -1209,7 +1209,7 @@
         <v>1772.888</v>
       </c>
       <c r="M8" t="n">
-        <v>108.2178545232641</v>
+        <v>208.3597497537472</v>
       </c>
       <c r="N8" t="n">
         <v>26.15586071767862</v>
@@ -1245,7 +1245,7 @@
         <v>714.4274</v>
       </c>
       <c r="Y8" t="n">
-        <v>73.92228427959083</v>
+        <v>142.3279801801077</v>
       </c>
       <c r="Z8" t="n">
         <v>9.2689338761061</v>
@@ -1308,7 +1308,7 @@
         <v>1888.707</v>
       </c>
       <c r="M9" t="n">
-        <v>109.7248753354082</v>
+        <v>211.2613271383233</v>
       </c>
       <c r="N9" t="n">
         <v>29.65123841101533</v>
@@ -1344,7 +1344,7 @@
         <v>665.6324</v>
       </c>
       <c r="Y9" t="n">
-        <v>70.97223581427968</v>
+        <v>136.6480361200311</v>
       </c>
       <c r="Z9" t="n">
         <v>9.008301684857699</v>
@@ -1407,7 +1407,7 @@
         <v>1963.644</v>
       </c>
       <c r="M10" t="n">
-        <v>109.4746178509552</v>
+        <v>210.7794881010929</v>
       </c>
       <c r="N10" t="n">
         <v>32.24423217187896</v>
@@ -1443,7 +1443,7 @@
         <v>635.0775</v>
       </c>
       <c r="Y10" t="n">
-        <v>69.18864744169888</v>
+        <v>133.2139629847635</v>
       </c>
       <c r="Z10" t="n">
         <v>8.637737840493624</v>
@@ -1506,7 +1506,7 @@
         <v>1970.661</v>
       </c>
       <c r="M11" t="n">
-        <v>106.7553373802408</v>
+        <v>205.5438585380755</v>
       </c>
       <c r="N11" t="n">
         <v>33.38365515560616</v>
@@ -1542,7 +1542,7 @@
         <v>574.5626999999999</v>
       </c>
       <c r="Y11" t="n">
-        <v>65.32181088310659</v>
+        <v>125.7688597600112</v>
       </c>
       <c r="Z11" t="n">
         <v>8.353255586685897</v>
@@ -1605,7 +1605,7 @@
         <v>1838.046</v>
       </c>
       <c r="M12" t="n">
-        <v>100.6382935248363</v>
+        <v>193.7662666373713</v>
       </c>
       <c r="N12" t="n">
         <v>31.04210160607312</v>
@@ -1641,7 +1641,7 @@
         <v>543.4535999999999</v>
       </c>
       <c r="Y12" t="n">
-        <v>61.61609472600434</v>
+        <v>118.63397342768</v>
       </c>
       <c r="Z12" t="n">
         <v>7.81562819139441</v>
@@ -1704,7 +1704,7 @@
         <v>1783.737</v>
       </c>
       <c r="M13" t="n">
-        <v>96.93582851694275</v>
+        <v>186.6376399803823</v>
       </c>
       <c r="N13" t="n">
         <v>30.86135953909287</v>
@@ -1740,7 +1740,7 @@
         <v>546.0051999999999</v>
       </c>
       <c r="Y13" t="n">
-        <v>59.72376574394802</v>
+        <v>114.9905340443179</v>
       </c>
       <c r="Z13" t="n">
         <v>7.498332516326033</v>
@@ -1759,996 +1759,6 @@
       </c>
       <c r="AE13" t="n">
         <v>-26.11900629581628</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>900</v>
-      </c>
-      <c r="D14" t="n">
-        <v>899.807285636</v>
-      </c>
-      <c r="E14" t="n">
-        <v>211.820965147</v>
-      </c>
-      <c r="F14" t="n">
-        <v>42.4165475698</v>
-      </c>
-      <c r="G14" t="n">
-        <v>49.72631602555686</v>
-      </c>
-      <c r="H14" t="n">
-        <v>268.5221065380071</v>
-      </c>
-      <c r="I14" t="n">
-        <v>1.267684274555436</v>
-      </c>
-      <c r="J14" t="n">
-        <v>818.1010032</v>
-      </c>
-      <c r="K14" t="n">
-        <v>3.862228663873061</v>
-      </c>
-      <c r="L14" t="n">
-        <v>1383.7706061</v>
-      </c>
-      <c r="M14" t="n">
-        <v>199.4328866534262</v>
-      </c>
-      <c r="N14" t="n">
-        <v>25.99995209197379</v>
-      </c>
-      <c r="O14" t="n">
-        <v>43.21582376606398</v>
-      </c>
-      <c r="P14" t="n">
-        <v>899.965</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>153.0359</v>
-      </c>
-      <c r="R14" t="n">
-        <v>59.591</v>
-      </c>
-      <c r="S14" t="n">
-        <v>73.66007416563659</v>
-      </c>
-      <c r="T14" t="n">
-        <v>154.6861557478368</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1.010783455044449</v>
-      </c>
-      <c r="V14" t="n">
-        <v>493.8484</v>
-      </c>
-      <c r="W14" t="n">
-        <v>3.227010132916525</v>
-      </c>
-      <c r="X14" t="n">
-        <v>626.0135</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>125.9094696987295</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>6.396908493687032</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>37.58201332579686</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>-113.8359507901702</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>-42.39351175135284</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>-0.256900819510987</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>-20.2653629667434</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D15" t="n">
-        <v>999.657661495</v>
-      </c>
-      <c r="E15" t="n">
-        <v>257.823580249</v>
-      </c>
-      <c r="F15" t="n">
-        <v>50.1537282104</v>
-      </c>
-      <c r="G15" t="n">
-        <v>58.79686777303634</v>
-      </c>
-      <c r="H15" t="n">
-        <v>317.5030859743962</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1.231474195136687</v>
-      </c>
-      <c r="J15" t="n">
-        <v>1066.51589024</v>
-      </c>
-      <c r="K15" t="n">
-        <v>4.136611124591413</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1808.42287132</v>
-      </c>
-      <c r="M15" t="n">
-        <v>237.7665274826089</v>
-      </c>
-      <c r="N15" t="n">
-        <v>39.21109490130724</v>
-      </c>
-      <c r="O15" t="n">
-        <v>44.48653525713356</v>
-      </c>
-      <c r="P15" t="n">
-        <v>999.899</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>182.1889</v>
-      </c>
-      <c r="R15" t="n">
-        <v>70.161</v>
-      </c>
-      <c r="S15" t="n">
-        <v>86.72558714462299</v>
-      </c>
-      <c r="T15" t="n">
-        <v>182.1237330037083</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0.9996423108307273</v>
-      </c>
-      <c r="V15" t="n">
-        <v>577.2861</v>
-      </c>
-      <c r="W15" t="n">
-        <v>3.168612906713856</v>
-      </c>
-      <c r="X15" t="n">
-        <v>696.9444</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>132.4059801264863</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>8.514083455979099</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>38.00086977651749</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>-135.379352970688</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>-42.63875185818039</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>-0.2318318843059595</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>-18.82555763015622</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D16" t="n">
-        <v>1099.76545523</v>
-      </c>
-      <c r="E16" t="n">
-        <v>285.693787152</v>
-      </c>
-      <c r="F16" t="n">
-        <v>55.1783532184</v>
-      </c>
-      <c r="G16" t="n">
-        <v>64.68740119390387</v>
-      </c>
-      <c r="H16" t="n">
-        <v>349.3119664470809</v>
-      </c>
-      <c r="I16" t="n">
-        <v>1.222679603673823</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1268.3126194</v>
-      </c>
-      <c r="K16" t="n">
-        <v>4.439412673420192</v>
-      </c>
-      <c r="L16" t="n">
-        <v>2068.45330718</v>
-      </c>
-      <c r="M16" t="n">
-        <v>260.4278275653932</v>
-      </c>
-      <c r="N16" t="n">
-        <v>49.21946241193401</v>
-      </c>
-      <c r="O16" t="n">
-        <v>44.80652170493985</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1100.059</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>236.6207</v>
-      </c>
-      <c r="R16" t="n">
-        <v>90.709</v>
-      </c>
-      <c r="S16" t="n">
-        <v>112.1248454882571</v>
-      </c>
-      <c r="T16" t="n">
-        <v>235.4621755253399</v>
-      </c>
-      <c r="U16" t="n">
-        <v>0.9951038752118473</v>
-      </c>
-      <c r="V16" t="n">
-        <v>732.7568</v>
-      </c>
-      <c r="W16" t="n">
-        <v>3.096756961669034</v>
-      </c>
-      <c r="X16" t="n">
-        <v>966.657</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>152.8105691663256</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>15.23641710058327</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>38.17418283984513</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>-113.849790921741</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>-32.5925825215005</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>-0.2275757284619757</v>
-      </c>
-      <c r="AE16" t="n">
-        <v>-18.61286699951254</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1200</v>
-      </c>
-      <c r="D17" t="n">
-        <v>1199.86290992</v>
-      </c>
-      <c r="E17" t="n">
-        <v>320.415589441</v>
-      </c>
-      <c r="F17" t="n">
-        <v>62.2541514527</v>
-      </c>
-      <c r="G17" t="n">
-        <v>72.98259255885112</v>
-      </c>
-      <c r="H17" t="n">
-        <v>394.1059998177961</v>
-      </c>
-      <c r="I17" t="n">
-        <v>1.229983848493006</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1394.40211569</v>
-      </c>
-      <c r="K17" t="n">
-        <v>4.351854783728491</v>
-      </c>
-      <c r="L17" t="n">
-        <v>2103.78106115</v>
-      </c>
-      <c r="M17" t="n">
-        <v>264.1959399479355</v>
-      </c>
-      <c r="N17" t="n">
-        <v>53.55340502049638</v>
-      </c>
-      <c r="O17" t="n">
-        <v>44.54043869545165</v>
-      </c>
-      <c r="P17" t="n">
-        <v>1199.668</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>261.7221</v>
-      </c>
-      <c r="R17" t="n">
-        <v>99.86499999999999</v>
-      </c>
-      <c r="S17" t="n">
-        <v>123.442521631644</v>
-      </c>
-      <c r="T17" t="n">
-        <v>259.2292954264524</v>
-      </c>
-      <c r="U17" t="n">
-        <v>0.9904753760819295</v>
-      </c>
-      <c r="V17" t="n">
-        <v>802.8339999999999</v>
-      </c>
-      <c r="W17" t="n">
-        <v>3.067505571749577</v>
-      </c>
-      <c r="X17" t="n">
-        <v>1003.726</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>153.3635080573405</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>17.74821902428575</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>38.35257109292667</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>-134.8767043913437</v>
-      </c>
-      <c r="AC17" t="n">
-        <v>-34.22345877852664</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>-0.2395084724110762</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>-19.47248922858016</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>1300</v>
-      </c>
-      <c r="D18" t="n">
-        <v>1299.7201242</v>
-      </c>
-      <c r="E18" t="n">
-        <v>346.076104124</v>
-      </c>
-      <c r="F18" t="n">
-        <v>67.6117271863</v>
-      </c>
-      <c r="G18" t="n">
-        <v>79.26345508358735</v>
-      </c>
-      <c r="H18" t="n">
-        <v>428.0226574513717</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1.236787667079175</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1501.12002116</v>
-      </c>
-      <c r="K18" t="n">
-        <v>4.337543110523877</v>
-      </c>
-      <c r="L18" t="n">
-        <v>2108.71964232</v>
-      </c>
-      <c r="M18" t="n">
-        <v>263.636130795378</v>
-      </c>
-      <c r="N18" t="n">
-        <v>57.08083544388736</v>
-      </c>
-      <c r="O18" t="n">
-        <v>44.29541275227747</v>
-      </c>
-      <c r="P18" t="n">
-        <v>1300.024</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>280.1731</v>
-      </c>
-      <c r="R18" t="n">
-        <v>107.281</v>
-      </c>
-      <c r="S18" t="n">
-        <v>132.6093943139679</v>
-      </c>
-      <c r="T18" t="n">
-        <v>278.4797280593326</v>
-      </c>
-      <c r="U18" t="n">
-        <v>0.9939559795688186</v>
-      </c>
-      <c r="V18" t="n">
-        <v>859.04</v>
-      </c>
-      <c r="W18" t="n">
-        <v>3.066104490402541</v>
-      </c>
-      <c r="X18" t="n">
-        <v>1003.352</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>151.3299523887224</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>19.44642153696666</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>38.21826927733208</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>-149.5429293920391</v>
-      </c>
-      <c r="AC18" t="n">
-        <v>-34.9380872224104</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>-0.2428316875103567</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>-19.63406443757911</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>1400</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1399.82352181</v>
-      </c>
-      <c r="E19" t="n">
-        <v>367.407812665</v>
-      </c>
-      <c r="F19" t="n">
-        <v>72.3903326484</v>
-      </c>
-      <c r="G19" t="n">
-        <v>84.8655716862837</v>
-      </c>
-      <c r="H19" t="n">
-        <v>458.274087105932</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1.247317208041472</v>
-      </c>
-      <c r="J19" t="n">
-        <v>1591.65581007</v>
-      </c>
-      <c r="K19" t="n">
-        <v>4.332122930443129</v>
-      </c>
-      <c r="L19" t="n">
-        <v>2087.90902829</v>
-      </c>
-      <c r="M19" t="n">
-        <v>261.1287621659193</v>
-      </c>
-      <c r="N19" t="n">
-        <v>59.57143091889137</v>
-      </c>
-      <c r="O19" t="n">
-        <v>43.92148191895775</v>
-      </c>
-      <c r="P19" t="n">
-        <v>1400.075</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>300.4143</v>
-      </c>
-      <c r="R19" t="n">
-        <v>115.281</v>
-      </c>
-      <c r="S19" t="n">
-        <v>142.4981458590853</v>
-      </c>
-      <c r="T19" t="n">
-        <v>299.2461063040791</v>
-      </c>
-      <c r="U19" t="n">
-        <v>0.9961113911823742</v>
-      </c>
-      <c r="V19" t="n">
-        <v>924.624</v>
-      </c>
-      <c r="W19" t="n">
-        <v>3.07782951743642</v>
-      </c>
-      <c r="X19" t="n">
-        <v>1029.969</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>151.4528223795006</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>21.8214326817</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>38.1355715969526</v>
-      </c>
-      <c r="AB19" t="n">
-        <v>-159.0279808018529</v>
-      </c>
-      <c r="AC19" t="n">
-        <v>-34.70149966500132</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>-0.251205816859098</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>-20.13968982706007</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D20" t="n">
-        <v>1499.6824457</v>
-      </c>
-      <c r="E20" t="n">
-        <v>388.694464627</v>
-      </c>
-      <c r="F20" t="n">
-        <v>77.63584094479999</v>
-      </c>
-      <c r="G20" t="n">
-        <v>91.01505386260257</v>
-      </c>
-      <c r="H20" t="n">
-        <v>491.4812908580539</v>
-      </c>
-      <c r="I20" t="n">
-        <v>1.264441188607331</v>
-      </c>
-      <c r="J20" t="n">
-        <v>1689.92398591</v>
-      </c>
-      <c r="K20" t="n">
-        <v>4.347692441495634</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2090.40048932</v>
-      </c>
-      <c r="M20" t="n">
-        <v>260.6430087969362</v>
-      </c>
-      <c r="N20" t="n">
-        <v>63.15925558260871</v>
-      </c>
-      <c r="O20" t="n">
-        <v>43.32666532362657</v>
-      </c>
-      <c r="P20" t="n">
-        <v>1500.016</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>301.1655</v>
-      </c>
-      <c r="R20" t="n">
-        <v>116.68</v>
-      </c>
-      <c r="S20" t="n">
-        <v>144.2274412855377</v>
-      </c>
-      <c r="T20" t="n">
-        <v>302.8776266996292</v>
-      </c>
-      <c r="U20" t="n">
-        <v>1.00568500276303</v>
-      </c>
-      <c r="V20" t="n">
-        <v>933.568</v>
-      </c>
-      <c r="W20" t="n">
-        <v>3.099850414473105</v>
-      </c>
-      <c r="X20" t="n">
-        <v>945.126</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>142.6978264604757</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>20.80657339648533</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>37.77254028111073</v>
-      </c>
-      <c r="AB20" t="n">
-        <v>-188.6036641584247</v>
-      </c>
-      <c r="AC20" t="n">
-        <v>-38.37453585041873</v>
-      </c>
-      <c r="AD20" t="n">
-        <v>-0.2587561858443008</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>-20.46407442083548</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>1600</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1599.77762091</v>
-      </c>
-      <c r="E21" t="n">
-        <v>394.333284808</v>
-      </c>
-      <c r="F21" t="n">
-        <v>79.76341055490001</v>
-      </c>
-      <c r="G21" t="n">
-        <v>93.50927380410317</v>
-      </c>
-      <c r="H21" t="n">
-        <v>504.9500785421571</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1.280515994961004</v>
-      </c>
-      <c r="J21" t="n">
-        <v>1757.33848801</v>
-      </c>
-      <c r="K21" t="n">
-        <v>4.456480230588814</v>
-      </c>
-      <c r="L21" t="n">
-        <v>2003.24394734</v>
-      </c>
-      <c r="M21" t="n">
-        <v>254.307230603555</v>
-      </c>
-      <c r="N21" t="n">
-        <v>65.04774618537127</v>
-      </c>
-      <c r="O21" t="n">
-        <v>42.7827691460166</v>
-      </c>
-      <c r="P21" t="n">
-        <v>1600.038</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>300.3554</v>
-      </c>
-      <c r="R21" t="n">
-        <v>117.308</v>
-      </c>
-      <c r="S21" t="n">
-        <v>145.0037082818294</v>
-      </c>
-      <c r="T21" t="n">
-        <v>304.5077873918418</v>
-      </c>
-      <c r="U21" t="n">
-        <v>1.013824913392074</v>
-      </c>
-      <c r="V21" t="n">
-        <v>939.66</v>
-      </c>
-      <c r="W21" t="n">
-        <v>3.12849377770468</v>
-      </c>
-      <c r="X21" t="n">
-        <v>871.4739999999999</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>134.7685023601441</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>19.76882940174999</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>37.46926789348365</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>-200.4422911503153</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>-39.69546687249021</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>-0.2666910815689301</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>-20.8268450076683</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1700</v>
-      </c>
-      <c r="D22" t="n">
-        <v>1699.63841723</v>
-      </c>
-      <c r="E22" t="n">
-        <v>392.44891672</v>
-      </c>
-      <c r="F22" t="n">
-        <v>79.86487850029999</v>
-      </c>
-      <c r="G22" t="n">
-        <v>93.62822801910902</v>
-      </c>
-      <c r="H22" t="n">
-        <v>505.5924313031887</v>
-      </c>
-      <c r="I22" t="n">
-        <v>1.288301253393223</v>
-      </c>
-      <c r="J22" t="n">
-        <v>1781.48985339</v>
-      </c>
-      <c r="K22" t="n">
-        <v>4.53941845037895</v>
-      </c>
-      <c r="L22" t="n">
-        <v>1872.93741169</v>
-      </c>
-      <c r="M22" t="n">
-        <v>241.8846982364728</v>
-      </c>
-      <c r="N22" t="n">
-        <v>64.1654884816061</v>
-      </c>
-      <c r="O22" t="n">
-        <v>42.52423108019509</v>
-      </c>
-      <c r="P22" t="n">
-        <v>1699.999</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>296.0968</v>
-      </c>
-      <c r="R22" t="n">
-        <v>117.119</v>
-      </c>
-      <c r="S22" t="n">
-        <v>144.770086526576</v>
-      </c>
-      <c r="T22" t="n">
-        <v>304.0171817058097</v>
-      </c>
-      <c r="U22" t="n">
-        <v>1.026749298559828</v>
-      </c>
-      <c r="V22" t="n">
-        <v>935.774</v>
-      </c>
-      <c r="W22" t="n">
-        <v>3.16036512383788</v>
-      </c>
-      <c r="X22" t="n">
-        <v>791.2596</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>126.3173259000818</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>18.32208567917583</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>36.99761697452185</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>-201.5752495973791</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>-39.86911929789162</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>-0.2615519548333953</v>
-      </c>
-      <c r="AE22" t="n">
-        <v>-20.30208028941215</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>sway_p8_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>SWay_P8_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1800</v>
-      </c>
-      <c r="D23" t="n">
-        <v>1799.73595333</v>
-      </c>
-      <c r="E23" t="n">
-        <v>394.618160262</v>
-      </c>
-      <c r="F23" t="n">
-        <v>81.3583114385</v>
-      </c>
-      <c r="G23" t="n">
-        <v>95.37902865005861</v>
-      </c>
-      <c r="H23" t="n">
-        <v>515.0467547103166</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1.305177527482162</v>
-      </c>
-      <c r="J23" t="n">
-        <v>1839.49337931</v>
-      </c>
-      <c r="K23" t="n">
-        <v>4.661451409354044</v>
-      </c>
-      <c r="L23" t="n">
-        <v>1824.85529229</v>
-      </c>
-      <c r="M23" t="n">
-        <v>236.7196328849409</v>
-      </c>
-      <c r="N23" t="n">
-        <v>66.41701487097963</v>
-      </c>
-      <c r="O23" t="n">
-        <v>41.97438206424157</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1799.979</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>291.8231</v>
-      </c>
-      <c r="R23" t="n">
-        <v>116.542</v>
-      </c>
-      <c r="S23" t="n">
-        <v>144.0568603213844</v>
-      </c>
-      <c r="T23" t="n">
-        <v>302.5194066749073</v>
-      </c>
-      <c r="U23" t="n">
-        <v>1.036653392671476</v>
-      </c>
-      <c r="V23" t="n">
-        <v>931.751</v>
-      </c>
-      <c r="W23" t="n">
-        <v>3.192862388207102</v>
-      </c>
-      <c r="X23" t="n">
-        <v>722.6549</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>118.9052406400124</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>16.99069460301212</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>36.64414503972399</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>-212.5273480354093</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>-41.26370006057864</v>
-      </c>
-      <c r="AD23" t="n">
-        <v>-0.2685241348106859</v>
-      </c>
-      <c r="AE23" t="n">
-        <v>-20.57376327408119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FPT torque and BMEP comparison plots
</commit_message>
<xml_diff>
--- a/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
+++ b/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AI23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,110 +464,130 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Diesel_Torque_Nm</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Diesel_BMEP_bar</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Diesel_Air_kg_h</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Diesel_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Diesel_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Diesel_Eta_v_pct</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Diesel_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>E94H6_Torque_Nm</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>E94H6_BMEP_bar</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>E94H6_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>E94H6_Eta_v_pct</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>E94H6_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -606,69 +626,81 @@
         <v>1.367320490870933</v>
       </c>
       <c r="J2" t="n">
+        <v>881.813</v>
+      </c>
+      <c r="K2" t="n">
+        <v>16.53908801576105</v>
+      </c>
+      <c r="L2" t="n">
         <v>414.5096</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>4.080967673971216</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>855.284</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>165.1217994474175</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>7.371469710110599</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>100.54</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>40.794</v>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
+        <v>872.4690000000001</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>16.36383403513333</v>
+      </c>
+      <c r="Z2" t="n">
         <v>343.2376</v>
       </c>
-      <c r="W2" t="n">
+      <c r="AA2" t="n">
         <v>3.413940720111398</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
         <v>614.033</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AC2" t="n">
         <v>138.4967160992609</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AD2" t="n">
         <v>5.123065851202532</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AE2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AF2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AG2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AH2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AI2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -705,69 +737,81 @@
         <v>1.349845689446515</v>
       </c>
       <c r="J3" t="n">
+        <v>898.116</v>
+      </c>
+      <c r="K3" t="n">
+        <v>16.84486344878478</v>
+      </c>
+      <c r="L3" t="n">
         <v>472.7576</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>4.189345630744473</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>1001.307</v>
       </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
         <v>173.5930765917979</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>9.478317989122266</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>43.955</v>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
+        <v>880.187</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>16.50859112229994</v>
+      </c>
+      <c r="Z3" t="n">
         <v>368.078</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AA3" t="n">
         <v>3.329561233304839</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AB3" t="n">
         <v>598.8225</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AC3" t="n">
         <v>135.9926355869658</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>5.277530107879249</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AF3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AG3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AH3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AI3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -804,69 +848,81 @@
         <v>1.320738085230403</v>
       </c>
       <c r="J4" t="n">
+        <v>929.991</v>
+      </c>
+      <c r="K4" t="n">
+        <v>17.44270384181866</v>
+      </c>
+      <c r="L4" t="n">
         <v>538.8533</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>4.255904799740311</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>1151.256</v>
       </c>
-      <c r="M4" t="n">
+      <c r="O4" t="n">
         <v>182.672058683661</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>12.20416552876442</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>47.414</v>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
+        <v>898.739</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>16.85654829787843</v>
+      </c>
+      <c r="Z4" t="n">
         <v>404.4934</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>3.303159897596289</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
         <v>618.6754</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AC4" t="n">
         <v>137.6591377994248</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AD4" t="n">
         <v>5.953061266356182</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AE4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AF4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AG4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AH4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AI4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -903,69 +959,81 @@
         <v>1.295256498794189</v>
       </c>
       <c r="J5" t="n">
+        <v>968.932</v>
+      </c>
+      <c r="K5" t="n">
+        <v>18.17307255539144</v>
+      </c>
+      <c r="L5" t="n">
         <v>611.21</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>4.302602003859044</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>1333.037</v>
       </c>
-      <c r="M5" t="n">
+      <c r="O5" t="n">
         <v>192.7045373690426</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>15.7296847843975</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>135.548</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>51.639</v>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="T5" t="n">
+      <c r="V5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="U5" t="n">
+      <c r="W5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
+        <v>924.303</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>17.33602098203586</v>
+      </c>
+      <c r="Z5" t="n">
         <v>439.0808</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>3.239301206952519</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
         <v>645.2624999999999</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AC5" t="n">
         <v>138.6621120271576</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AD5" t="n">
         <v>6.691189980673633</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AE5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AF5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AG5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AH5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AI5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -1002,69 +1070,81 @@
         <v>1.314863921205991</v>
       </c>
       <c r="J6" t="n">
+        <v>1009.037</v>
+      </c>
+      <c r="K6" t="n">
+        <v>18.92527299343453</v>
+      </c>
+      <c r="L6" t="n">
         <v>717.2952</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>4.525441821847942</v>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>1638.823</v>
       </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
         <v>211.2164884552933</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>22.0044045378286</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>58.213</v>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
+        <v>977.721</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>18.33791707976398</v>
+      </c>
+      <c r="Z6" t="n">
         <v>493.4668</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>3.211861058625126</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
         <v>706.9007</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AC6" t="n">
         <v>145.520665121553</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AD6" t="n">
         <v>8.086896229873149</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AE6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AF6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AG6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AH6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AI6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -1101,69 +1181,81 @@
         <v>1.30800901886618</v>
       </c>
       <c r="J7" t="n">
+        <v>1002.874</v>
+      </c>
+      <c r="K7" t="n">
+        <v>18.80968113955946</v>
+      </c>
+      <c r="L7" t="n">
         <v>759.0008</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>4.516775727741662</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>1713.213</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>209.4446160066526</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>24.09184179296887</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>62.66</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
+        <v>988.704</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>18.54391177895428</v>
+      </c>
+      <c r="Z7" t="n">
         <v>522.3481</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AA7" t="n">
         <v>3.153700834751151</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
         <v>720.8134</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AC7" t="n">
         <v>144.0517827851469</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AD7" t="n">
         <v>8.844545266070686</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AE7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AF7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AG7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AH7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AI7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -1200,69 +1292,81 @@
         <v>1.306559021984483</v>
       </c>
       <c r="J8" t="n">
+        <v>1004.717</v>
+      </c>
+      <c r="K8" t="n">
+        <v>18.84424803663747</v>
+      </c>
+      <c r="L8" t="n">
         <v>802.591</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>4.487202997614924</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>1772.888</v>
       </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
         <v>208.3597497537472</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>26.15586071767862</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>65.848</v>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="T8" t="n">
+      <c r="V8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="U8" t="n">
+      <c r="W8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
+        <v>978.561</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>18.35367193247452</v>
+      </c>
+      <c r="Z8" t="n">
         <v>548.4717000000001</v>
       </c>
-      <c r="W8" t="n">
+      <c r="AA8" t="n">
         <v>3.14799857887937</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AB8" t="n">
         <v>714.4274</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AC8" t="n">
         <v>142.3279801801077</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AD8" t="n">
         <v>9.2689338761061</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AE8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AF8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AG8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AH8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AI8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1299,69 +1403,81 @@
         <v>1.316127269014794</v>
       </c>
       <c r="J9" t="n">
+        <v>1005.259</v>
+      </c>
+      <c r="K9" t="n">
+        <v>18.85441366779117</v>
+      </c>
+      <c r="L9" t="n">
         <v>861.736</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>4.547873112410683</v>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>1888.707</v>
       </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
         <v>211.2613271383233</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>29.65123841101533</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="S9" t="n">
+      <c r="U9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="T9" t="n">
+      <c r="V9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="U9" t="n">
+      <c r="W9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
+        <v>938.7430000000001</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>17.60685440244086</v>
+      </c>
+      <c r="Z9" t="n">
         <v>558.4708000000001</v>
       </c>
-      <c r="W9" t="n">
+      <c r="AA9" t="n">
         <v>3.157496350455755</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AB9" t="n">
         <v>665.6324</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AC9" t="n">
         <v>136.6480361200311</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AD9" t="n">
         <v>9.008301684857699</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AE9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AF9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AG9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AH9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AI9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1398,69 +1514,81 @@
         <v>1.326501688644143</v>
       </c>
       <c r="J10" t="n">
+        <v>1002.887</v>
+      </c>
+      <c r="K10" t="n">
+        <v>18.80992496466094</v>
+      </c>
+      <c r="L10" t="n">
         <v>906.6950000000001</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>4.543734753072438</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>1963.644</v>
       </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
         <v>210.7794881010929</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>32.24423217187896</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>180.749</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>68.246</v>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="T10" t="n">
+      <c r="V10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="U10" t="n">
+      <c r="W10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
+        <v>907.992</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>17.03009550279584</v>
+      </c>
+      <c r="Z10" t="n">
         <v>571.497</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AA10" t="n">
         <v>3.161826621447422</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AB10" t="n">
         <v>635.0775</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AC10" t="n">
         <v>133.2139629847635</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AD10" t="n">
         <v>8.637737840493624</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AE10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AF10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AG10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AH10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AI10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1497,69 +1625,81 @@
         <v>1.346265262913802</v>
       </c>
       <c r="J11" t="n">
+        <v>983.236</v>
+      </c>
+      <c r="K11" t="n">
+        <v>18.44135519011949</v>
+      </c>
+      <c r="L11" t="n">
         <v>931.8920000000001</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>4.525500655108144</v>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>1970.661</v>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>205.5438585380755</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>33.38365515560616</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>67.595</v>
       </c>
-      <c r="S11" t="n">
+      <c r="U11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="T11" t="n">
+      <c r="V11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="U11" t="n">
+      <c r="W11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
+        <v>860.047</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>16.13084977278771</v>
+      </c>
+      <c r="Z11" t="n">
         <v>572.1528</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AA11" t="n">
         <v>3.174929637488791</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AB11" t="n">
         <v>574.5626999999999</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AC11" t="n">
         <v>125.7688597600112</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AD11" t="n">
         <v>8.353255586685897</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AE11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AF11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AG11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AH11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AI11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1596,69 +1736,81 @@
         <v>1.342323063096884</v>
       </c>
       <c r="J12" t="n">
+        <v>867.4299999999999</v>
+      </c>
+      <c r="K12" t="n">
+        <v>16.26932367464713</v>
+      </c>
+      <c r="L12" t="n">
         <v>920.961</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>4.828357974205725</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>1838.046</v>
       </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
         <v>193.7662666373713</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>31.04210160607312</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="R12" t="n">
+      <c r="T12" t="n">
         <v>67.64</v>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="T12" t="n">
+      <c r="V12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="U12" t="n">
+      <c r="W12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
+        <v>801.8111</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>15.03859021687613</v>
+      </c>
+      <c r="Z12" t="n">
         <v>566.0339</v>
       </c>
-      <c r="W12" t="n">
+      <c r="AA12" t="n">
         <v>3.209340208243088</v>
       </c>
-      <c r="X12" t="n">
+      <c r="AB12" t="n">
         <v>543.4535999999999</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AC12" t="n">
         <v>118.63397342768</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AD12" t="n">
         <v>7.81562819139441</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AE12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AF12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AG12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AH12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AI12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -1695,70 +1847,1192 @@
         <v>1.371245975843687</v>
       </c>
       <c r="J13" t="n">
+        <v>781.862</v>
+      </c>
+      <c r="K13" t="n">
+        <v>14.66442934520014</v>
+      </c>
+      <c r="L13" t="n">
         <v>930.189</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>5.164285285998859</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>1783.737</v>
       </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
         <v>186.6376399803823</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>30.86135953909287</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="R13" t="n">
+      <c r="T13" t="n">
         <v>68.863</v>
       </c>
-      <c r="S13" t="n">
+      <c r="U13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="T13" t="n">
+      <c r="V13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="U13" t="n">
+      <c r="W13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="V13" t="n">
+      <c r="X13" t="n">
+        <v>765.7402</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>14.36205245897539</v>
+      </c>
+      <c r="Z13" t="n">
         <v>570.3287</v>
       </c>
-      <c r="W13" t="n">
+      <c r="AA13" t="n">
         <v>3.232336817144408</v>
       </c>
-      <c r="X13" t="n">
+      <c r="AB13" t="n">
         <v>546.0051999999999</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AC13" t="n">
         <v>114.9905340443179</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AD13" t="n">
         <v>7.498332516326033</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AE13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AF13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AG13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AH13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AI13" t="n">
         <v>-26.11900629581628</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>900</v>
+      </c>
+      <c r="D14" t="n">
+        <v>899.807285636</v>
+      </c>
+      <c r="E14" t="n">
+        <v>211.820965147</v>
+      </c>
+      <c r="F14" t="n">
+        <v>42.4165475698</v>
+      </c>
+      <c r="G14" t="n">
+        <v>49.72631602555686</v>
+      </c>
+      <c r="H14" t="n">
+        <v>268.5221065380071</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1.267684274555436</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2247.96135288</v>
+      </c>
+      <c r="K14" t="n">
+        <v>21.89822905972583</v>
+      </c>
+      <c r="L14" t="n">
+        <v>818.1010032</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3.862228663873061</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1383.7706061</v>
+      </c>
+      <c r="O14" t="n">
+        <v>199.4328866534262</v>
+      </c>
+      <c r="P14" t="n">
+        <v>25.99995209197379</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>43.21582376606398</v>
+      </c>
+      <c r="R14" t="n">
+        <v>899.965</v>
+      </c>
+      <c r="S14" t="n">
+        <v>153.0359</v>
+      </c>
+      <c r="T14" t="n">
+        <v>59.591</v>
+      </c>
+      <c r="U14" t="n">
+        <v>73.66007416563659</v>
+      </c>
+      <c r="V14" t="n">
+        <v>154.6861557478368</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1.010783455044449</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1633.001</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>15.90767114699158</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>493.8484</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>3.227010132916525</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>626.0135</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>125.9094696987295</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>6.396908493687032</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>37.58201332579686</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>-113.8359507901702</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>-42.39351175135284</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>-0.256900819510987</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>-20.2653629667434</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D15" t="n">
+        <v>999.657661495</v>
+      </c>
+      <c r="E15" t="n">
+        <v>257.823580249</v>
+      </c>
+      <c r="F15" t="n">
+        <v>50.1537282104</v>
+      </c>
+      <c r="G15" t="n">
+        <v>58.79686777303634</v>
+      </c>
+      <c r="H15" t="n">
+        <v>317.5030859743962</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.231474195136687</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2462.87816125</v>
+      </c>
+      <c r="K15" t="n">
+        <v>23.99181376145656</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1066.51589024</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4.136611124591413</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1808.42287132</v>
+      </c>
+      <c r="O15" t="n">
+        <v>237.7665274826089</v>
+      </c>
+      <c r="P15" t="n">
+        <v>39.21109490130724</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>44.48653525713356</v>
+      </c>
+      <c r="R15" t="n">
+        <v>999.899</v>
+      </c>
+      <c r="S15" t="n">
+        <v>182.1889</v>
+      </c>
+      <c r="T15" t="n">
+        <v>70.161</v>
+      </c>
+      <c r="U15" t="n">
+        <v>86.72558714462299</v>
+      </c>
+      <c r="V15" t="n">
+        <v>182.1237330037083</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.9996423108307273</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1744.402</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>16.9928697925809</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>577.2861</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>3.168612906713856</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>696.9444</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>132.4059801264863</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>8.514083455979099</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>38.00086977651749</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>-135.379352970688</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>-42.63875185818039</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>-0.2318318843059595</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>-18.82555763015622</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1099.76545523</v>
+      </c>
+      <c r="E16" t="n">
+        <v>285.693787152</v>
+      </c>
+      <c r="F16" t="n">
+        <v>55.1783532184</v>
+      </c>
+      <c r="G16" t="n">
+        <v>64.68740119390387</v>
+      </c>
+      <c r="H16" t="n">
+        <v>349.3119664470809</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.222679603673823</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2480.66514028</v>
+      </c>
+      <c r="K16" t="n">
+        <v>24.16508335106959</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1268.3126194</v>
+      </c>
+      <c r="M16" t="n">
+        <v>4.439412673420192</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2068.45330718</v>
+      </c>
+      <c r="O16" t="n">
+        <v>260.4278275653932</v>
+      </c>
+      <c r="P16" t="n">
+        <v>49.21946241193401</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>44.80652170493985</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1100.059</v>
+      </c>
+      <c r="S16" t="n">
+        <v>236.6207</v>
+      </c>
+      <c r="T16" t="n">
+        <v>90.709</v>
+      </c>
+      <c r="U16" t="n">
+        <v>112.1248454882571</v>
+      </c>
+      <c r="V16" t="n">
+        <v>235.4621755253399</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.9951038752118473</v>
+      </c>
+      <c r="X16" t="n">
+        <v>2059.023</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>20.05771017169742</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>732.7568</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>3.096756961669034</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>966.657</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>152.8105691663256</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>15.23641710058327</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>38.17418283984513</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>-113.849790921741</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>-32.5925825215005</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>-0.2275757284619757</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>-18.61286699951254</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1199.86290992</v>
+      </c>
+      <c r="E17" t="n">
+        <v>320.415589441</v>
+      </c>
+      <c r="F17" t="n">
+        <v>62.2541514527</v>
+      </c>
+      <c r="G17" t="n">
+        <v>72.98259255885112</v>
+      </c>
+      <c r="H17" t="n">
+        <v>394.1059998177961</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1.229983848493006</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2550.09139118</v>
+      </c>
+      <c r="K17" t="n">
+        <v>24.84139032717415</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1394.40211569</v>
+      </c>
+      <c r="M17" t="n">
+        <v>4.351854783728491</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2103.78106115</v>
+      </c>
+      <c r="O17" t="n">
+        <v>264.1959399479355</v>
+      </c>
+      <c r="P17" t="n">
+        <v>53.55340502049638</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>44.54043869545165</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1199.668</v>
+      </c>
+      <c r="S17" t="n">
+        <v>261.7221</v>
+      </c>
+      <c r="T17" t="n">
+        <v>99.86499999999999</v>
+      </c>
+      <c r="U17" t="n">
+        <v>123.442521631644</v>
+      </c>
+      <c r="V17" t="n">
+        <v>259.2292954264524</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.9904753760819295</v>
+      </c>
+      <c r="X17" t="n">
+        <v>2087.014</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>20.33038093128387</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>802.8339999999999</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>3.067505571749577</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>1003.726</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>153.3635080573405</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>17.74821902428575</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>38.35257109292667</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>-134.8767043913437</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>-34.22345877852664</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>-0.2395084724110762</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>-19.47248922858016</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1299.7201242</v>
+      </c>
+      <c r="E18" t="n">
+        <v>346.076104124</v>
+      </c>
+      <c r="F18" t="n">
+        <v>67.6117271863</v>
+      </c>
+      <c r="G18" t="n">
+        <v>79.26345508358735</v>
+      </c>
+      <c r="H18" t="n">
+        <v>428.0226574513717</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.236787667079175</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2542.651754</v>
+      </c>
+      <c r="K18" t="n">
+        <v>24.76891804962357</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1501.12002116</v>
+      </c>
+      <c r="M18" t="n">
+        <v>4.337543110523877</v>
+      </c>
+      <c r="N18" t="n">
+        <v>2108.71964232</v>
+      </c>
+      <c r="O18" t="n">
+        <v>263.636130795378</v>
+      </c>
+      <c r="P18" t="n">
+        <v>57.08083544388736</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>44.29541275227747</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1300.024</v>
+      </c>
+      <c r="S18" t="n">
+        <v>280.1731</v>
+      </c>
+      <c r="T18" t="n">
+        <v>107.281</v>
+      </c>
+      <c r="U18" t="n">
+        <v>132.6093943139679</v>
+      </c>
+      <c r="V18" t="n">
+        <v>278.4797280593326</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.9939559795688186</v>
+      </c>
+      <c r="X18" t="n">
+        <v>2062.997</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>20.0964223862877</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>859.04</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>3.066104490402541</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>1003.352</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>151.3299523887224</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>19.44642153696666</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>38.21826927733208</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>-149.5429293920391</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>-34.9380872224104</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>-0.2428316875103567</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>-19.63406443757911</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1400</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1399.82352181</v>
+      </c>
+      <c r="E19" t="n">
+        <v>367.407812665</v>
+      </c>
+      <c r="F19" t="n">
+        <v>72.3903326484</v>
+      </c>
+      <c r="G19" t="n">
+        <v>84.8655716862837</v>
+      </c>
+      <c r="H19" t="n">
+        <v>458.274087105932</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1.247317208041472</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2506.42407501</v>
+      </c>
+      <c r="K19" t="n">
+        <v>24.41601073126204</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1591.65581007</v>
+      </c>
+      <c r="M19" t="n">
+        <v>4.332122930443129</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2087.90902829</v>
+      </c>
+      <c r="O19" t="n">
+        <v>261.1287621659193</v>
+      </c>
+      <c r="P19" t="n">
+        <v>59.57143091889137</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>43.92148191895775</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1400.075</v>
+      </c>
+      <c r="S19" t="n">
+        <v>300.4143</v>
+      </c>
+      <c r="T19" t="n">
+        <v>115.281</v>
+      </c>
+      <c r="U19" t="n">
+        <v>142.4981458590853</v>
+      </c>
+      <c r="V19" t="n">
+        <v>299.2461063040791</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.9961113911823742</v>
+      </c>
+      <c r="X19" t="n">
+        <v>2052.946</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>19.99851185059396</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>924.624</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>3.07782951743642</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>1029.969</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>151.4528223795006</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>21.8214326817</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>38.1355715969526</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>-159.0279808018529</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>-34.70149966500132</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>-0.251205816859098</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>-20.13968982706007</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1499.6824457</v>
+      </c>
+      <c r="E20" t="n">
+        <v>388.694464627</v>
+      </c>
+      <c r="F20" t="n">
+        <v>77.63584094479999</v>
+      </c>
+      <c r="G20" t="n">
+        <v>91.01505386260257</v>
+      </c>
+      <c r="H20" t="n">
+        <v>491.4812908580539</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1.264441188607331</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2475.06577227</v>
+      </c>
+      <c r="K20" t="n">
+        <v>24.11053782113172</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1689.92398591</v>
+      </c>
+      <c r="M20" t="n">
+        <v>4.347692441495634</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2090.40048932</v>
+      </c>
+      <c r="O20" t="n">
+        <v>260.6430087969362</v>
+      </c>
+      <c r="P20" t="n">
+        <v>63.15925558260871</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>43.32666532362657</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1500.016</v>
+      </c>
+      <c r="S20" t="n">
+        <v>301.1655</v>
+      </c>
+      <c r="T20" t="n">
+        <v>116.68</v>
+      </c>
+      <c r="U20" t="n">
+        <v>144.2274412855377</v>
+      </c>
+      <c r="V20" t="n">
+        <v>302.8776266996292</v>
+      </c>
+      <c r="W20" t="n">
+        <v>1.00568500276303</v>
+      </c>
+      <c r="X20" t="n">
+        <v>1920.083</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>18.70424386692295</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>933.568</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>3.099850414473105</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>945.126</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>142.6978264604757</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>20.80657339648533</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>37.77254028111073</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>-188.6036641584247</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>-38.37453585041873</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>-0.2587561858443008</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>-20.46407442083548</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1599.77762091</v>
+      </c>
+      <c r="E21" t="n">
+        <v>394.333284808</v>
+      </c>
+      <c r="F21" t="n">
+        <v>79.76341055490001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>93.50927380410317</v>
+      </c>
+      <c r="H21" t="n">
+        <v>504.9500785421571</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1.280515994961004</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2353.82949239</v>
+      </c>
+      <c r="K21" t="n">
+        <v>22.92953004990827</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1757.33848801</v>
+      </c>
+      <c r="M21" t="n">
+        <v>4.456480230588814</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2003.24394734</v>
+      </c>
+      <c r="O21" t="n">
+        <v>254.307230603555</v>
+      </c>
+      <c r="P21" t="n">
+        <v>65.04774618537127</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>42.7827691460166</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1600.038</v>
+      </c>
+      <c r="S21" t="n">
+        <v>300.3554</v>
+      </c>
+      <c r="T21" t="n">
+        <v>117.308</v>
+      </c>
+      <c r="U21" t="n">
+        <v>145.0037082818294</v>
+      </c>
+      <c r="V21" t="n">
+        <v>304.5077873918418</v>
+      </c>
+      <c r="W21" t="n">
+        <v>1.013824913392074</v>
+      </c>
+      <c r="X21" t="n">
+        <v>1795.378</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>17.48944600067205</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>939.66</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>3.12849377770468</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>871.4739999999999</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>134.7685023601441</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>19.76882940174999</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>37.46926789348365</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>-200.4422911503153</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>-39.69546687249021</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>-0.2666910815689301</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>-20.8268450076683</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1699.63841723</v>
+      </c>
+      <c r="E22" t="n">
+        <v>392.44891672</v>
+      </c>
+      <c r="F22" t="n">
+        <v>79.86487850029999</v>
+      </c>
+      <c r="G22" t="n">
+        <v>93.62822801910902</v>
+      </c>
+      <c r="H22" t="n">
+        <v>505.5924313031887</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.288301253393223</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2204.98225505</v>
+      </c>
+      <c r="K22" t="n">
+        <v>21.47955365507267</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1781.48985339</v>
+      </c>
+      <c r="M22" t="n">
+        <v>4.53941845037895</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1872.93741169</v>
+      </c>
+      <c r="O22" t="n">
+        <v>241.8846982364728</v>
+      </c>
+      <c r="P22" t="n">
+        <v>64.1654884816061</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>42.52423108019509</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1699.999</v>
+      </c>
+      <c r="S22" t="n">
+        <v>296.0968</v>
+      </c>
+      <c r="T22" t="n">
+        <v>117.119</v>
+      </c>
+      <c r="U22" t="n">
+        <v>144.770086526576</v>
+      </c>
+      <c r="V22" t="n">
+        <v>304.0171817058097</v>
+      </c>
+      <c r="W22" t="n">
+        <v>1.026749298559828</v>
+      </c>
+      <c r="X22" t="n">
+        <v>1665.875</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>16.22790902883379</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>935.774</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>3.16036512383788</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>791.2596</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>126.3173259000818</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>18.32208567917583</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>36.99761697452185</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>-201.5752495973791</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>-39.86911929789162</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>-0.2615519548333953</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>-20.30208028941215</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sway_p8_c13_full_load_curve_brazil_397kw_d85b15__vs__p251191_c13_etanol_full_load_curve_rev_26</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SWay_P8_C13_Full Load Curve_Brazil_397kW_D85B15 vs P251191_C13_Etanol_Full_Load_Curve_Rev_26</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1799.73595333</v>
+      </c>
+      <c r="E23" t="n">
+        <v>394.618160262</v>
+      </c>
+      <c r="F23" t="n">
+        <v>81.3583114385</v>
+      </c>
+      <c r="G23" t="n">
+        <v>95.37902865005861</v>
+      </c>
+      <c r="H23" t="n">
+        <v>515.0467547103166</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.305177527482162</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2093.79388149</v>
+      </c>
+      <c r="K23" t="n">
+        <v>20.39642628285346</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1839.49337931</v>
+      </c>
+      <c r="M23" t="n">
+        <v>4.661451409354044</v>
+      </c>
+      <c r="N23" t="n">
+        <v>1824.85529229</v>
+      </c>
+      <c r="O23" t="n">
+        <v>236.7196328849409</v>
+      </c>
+      <c r="P23" t="n">
+        <v>66.41701487097963</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>41.97438206424157</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1799.979</v>
+      </c>
+      <c r="S23" t="n">
+        <v>291.8231</v>
+      </c>
+      <c r="T23" t="n">
+        <v>116.542</v>
+      </c>
+      <c r="U23" t="n">
+        <v>144.0568603213844</v>
+      </c>
+      <c r="V23" t="n">
+        <v>302.5194066749073</v>
+      </c>
+      <c r="W23" t="n">
+        <v>1.036653392671476</v>
+      </c>
+      <c r="X23" t="n">
+        <v>1551.491</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>15.11365186887033</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>931.751</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>3.192862388207102</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>722.6549</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>118.9052406400124</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>16.99069460301212</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>36.64414503972399</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>-212.5273480354093</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>-41.26370006057864</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>-0.2685241348106859</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>-20.57376327408119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix SWay compressor inlet pressure conversion
</commit_message>
<xml_diff>
--- a/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
+++ b/out_FPT/compare_rpm_diesel_vs_e94h6_fpt.xlsx
@@ -2133,8 +2133,12 @@
       <c r="M14" t="n">
         <v>3.862228663873061</v>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>2.394947865647763</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.1906927639437788</v>
+      </c>
       <c r="P14" t="n">
         <v>1383.7706061</v>
       </c>
@@ -2252,8 +2256,12 @@
       <c r="M15" t="n">
         <v>4.136611124591413</v>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>2.847439177810685</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.2506917189847213</v>
+      </c>
       <c r="P15" t="n">
         <v>1808.42287132</v>
       </c>
@@ -2371,8 +2379,12 @@
       <c r="M16" t="n">
         <v>4.439412673420192</v>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>3.139663848283791</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.3006765122493675</v>
+      </c>
       <c r="P16" t="n">
         <v>2068.45330718</v>
       </c>
@@ -2490,8 +2502,12 @@
       <c r="M17" t="n">
         <v>4.351854783728491</v>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>3.201759989156442</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.3326502254066982</v>
+      </c>
       <c r="P17" t="n">
         <v>2103.78106115</v>
       </c>
@@ -2609,8 +2625,12 @@
       <c r="M18" t="n">
         <v>4.337543110523877</v>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>3.236706916900525</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.3601964987750724</v>
+      </c>
       <c r="P18" t="n">
         <v>2108.71964232</v>
       </c>
@@ -2728,8 +2748,12 @@
       <c r="M19" t="n">
         <v>4.332122930443129</v>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>3.241943089107858</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.3841165943639843</v>
+      </c>
       <c r="P19" t="n">
         <v>2087.90902829</v>
       </c>
@@ -2847,8 +2871,12 @@
       <c r="M20" t="n">
         <v>4.347692441495634</v>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>3.278674470393804</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.4104028682278533</v>
+      </c>
       <c r="P20" t="n">
         <v>2090.40048932</v>
       </c>
@@ -2966,8 +2994,12 @@
       <c r="M21" t="n">
         <v>4.456480230588814</v>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>3.209033350920502</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.4285883475937811</v>
+      </c>
       <c r="P21" t="n">
         <v>2003.24394734</v>
       </c>
@@ -3085,8 +3117,12 @@
       <c r="M22" t="n">
         <v>4.53941845037895</v>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>3.083141085728647</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.4353538353188192</v>
+      </c>
       <c r="P22" t="n">
         <v>1872.93741169</v>
       </c>
@@ -3204,8 +3240,12 @@
       <c r="M23" t="n">
         <v>4.661451409354044</v>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>3.052200566203288</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.4512066176176181</v>
+      </c>
       <c r="P23" t="n">
         <v>1824.85529229</v>
       </c>

</xml_diff>